<commit_message>
chore: guardar todos los cambios locales y sincronizar repositorio
</commit_message>
<xml_diff>
--- a/puestos_votacion_prueba.xlsx
+++ b/puestos_votacion_prueba.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\richb\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\RICHARD\RB\2027\Proyecto Elecciones 2027\Soacha\Pruebas Puestos de Votacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6E6331E-ABBD-40A7-AFF6-A9AC44F5AFC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D53E9BA2-C336-475E-9CD6-DA5BF0E9BCCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="990" uniqueCount="373">
   <si>
     <t>NUIP</t>
   </si>
@@ -1055,6 +1055,111 @@
   </si>
   <si>
     <t>P50</t>
+  </si>
+  <si>
+    <t>CC GRAN PLAZA BOSA</t>
+  </si>
+  <si>
+    <t>CLL 65 SUR No 78H-51</t>
+  </si>
+  <si>
+    <t>P69</t>
+  </si>
+  <si>
+    <t>CEDID SAN PABLO</t>
+  </si>
+  <si>
+    <t>CRA 77L No 65J - 73 SUR</t>
+  </si>
+  <si>
+    <t>P70</t>
+  </si>
+  <si>
+    <t>VILLA DEL RIO</t>
+  </si>
+  <si>
+    <t>CLL 55A SUR No 66-50</t>
+  </si>
+  <si>
+    <t>P71</t>
+  </si>
+  <si>
+    <t>I E JULIO CESAR TURBAY AYALA</t>
+  </si>
+  <si>
+    <t>TV 9 ESTE No 45A- 80</t>
+  </si>
+  <si>
+    <t>I.E. COMPARTIR PRIMARIA</t>
+  </si>
+  <si>
+    <t>CR. 15 A NO. 5 C - 16 SUR</t>
+  </si>
+  <si>
+    <t>P66</t>
+  </si>
+  <si>
+    <t>I. E. SANTA ANA - ANTONIO NARIÑO</t>
+  </si>
+  <si>
+    <t>CR. 11 D No. 17 A - 44 SUR SANTA ANA</t>
+  </si>
+  <si>
+    <t>P67</t>
+  </si>
+  <si>
+    <t>CENTRO COMERCIAL GRAN PLAZA</t>
+  </si>
+  <si>
+    <t>CRA 7 No 30B - 139</t>
+  </si>
+  <si>
+    <t>P68</t>
+  </si>
+  <si>
+    <t>COLEGIO DEL PILAR</t>
+  </si>
+  <si>
+    <t>CLL 62 No 27A-12</t>
+  </si>
+  <si>
+    <t>P72</t>
+  </si>
+  <si>
+    <t>PIAMONTE</t>
+  </si>
+  <si>
+    <t>CLL 68A SUR No 80H-05</t>
+  </si>
+  <si>
+    <t>P73</t>
+  </si>
+  <si>
+    <t>COL GABRIEL BETANCOURT MEJIA</t>
+  </si>
+  <si>
+    <t>CRA 87A No 6A-23 Y CRA 88 No 6A-28</t>
+  </si>
+  <si>
+    <t>P74</t>
+  </si>
+  <si>
+    <t>UNIVER. DE CUNDINAMARCA EXTENSION SOACHA</t>
+  </si>
+  <si>
+    <t>DIAG. 9 No. 4 B - 85</t>
+  </si>
+  <si>
+    <t>P75</t>
+  </si>
+  <si>
+    <t>LA CABAÑA</t>
+  </si>
+  <si>
+    <t>CLL 63 B # 71A-18</t>
+  </si>
+  <si>
+    <t>P76</t>
   </si>
 </sst>
 </file>
@@ -1457,7 +1562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -4970,6 +5075,728 @@
       </c>
       <c r="L81" s="3" t="s">
         <v>337</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A82" s="2">
+        <v>80126131</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="E82" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="F82" s="3">
+        <v>6</v>
+      </c>
+      <c r="G82" s="5">
+        <v>4.6200999999999999</v>
+      </c>
+      <c r="H82" s="5">
+        <v>-74.192300000000003</v>
+      </c>
+      <c r="I82" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J82" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K82" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L82" s="3" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A83" s="2">
+        <v>52243197</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="E83" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="F83" s="3">
+        <v>4</v>
+      </c>
+      <c r="G83" s="5">
+        <v>4.6062000000000003</v>
+      </c>
+      <c r="H83" s="5">
+        <v>-74.178399999999996</v>
+      </c>
+      <c r="I83" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J83" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K83" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L83" s="3" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A84" s="2">
+        <v>1024508725</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="E84" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="F84" s="3">
+        <v>18</v>
+      </c>
+      <c r="G84" s="5">
+        <v>4.5881616000000003</v>
+      </c>
+      <c r="H84" s="5">
+        <v>-74.203519099999994</v>
+      </c>
+      <c r="I84" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J84" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K84" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L84" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A85" s="2">
+        <v>1032417059</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="F85" s="3">
+        <v>24</v>
+      </c>
+      <c r="G85" s="5">
+        <v>4.6151999999999997</v>
+      </c>
+      <c r="H85" s="5">
+        <v>-74.148499999999999</v>
+      </c>
+      <c r="I85" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J85" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K85" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L85" s="3" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A86" s="2">
+        <v>53099030</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D86" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="E86" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="F86" s="3">
+        <v>8</v>
+      </c>
+      <c r="G86" s="5">
+        <v>4.5954600000000001</v>
+      </c>
+      <c r="H86" s="5">
+        <v>-74.19502</v>
+      </c>
+      <c r="I86" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J86" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K86" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L86" s="3" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A87" s="2">
+        <v>1012434961</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="F87" s="3">
+        <v>17</v>
+      </c>
+      <c r="G87" s="5">
+        <v>4.58256</v>
+      </c>
+      <c r="H87" s="5">
+        <v>-74.194387000000006</v>
+      </c>
+      <c r="I87" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J87" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K87" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L87" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A88" s="2">
+        <v>1073711749</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D88" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="E88" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="F88" s="3">
+        <v>29</v>
+      </c>
+      <c r="G88" s="5">
+        <v>4.5682999999999998</v>
+      </c>
+      <c r="H88" s="5">
+        <v>-74.234300000000005</v>
+      </c>
+      <c r="I88" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J88" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K88" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L88" s="3" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A89" s="2">
+        <v>80828793</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="F89" s="3">
+        <v>14</v>
+      </c>
+      <c r="G89" s="5">
+        <v>4.5686</v>
+      </c>
+      <c r="H89" s="5">
+        <v>-74.225499999999997</v>
+      </c>
+      <c r="I89" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J89" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K89" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L89" s="3" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A90" s="2">
+        <v>21118151</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="E90" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="F90" s="3">
+        <v>3</v>
+      </c>
+      <c r="G90" s="5">
+        <v>4.5865999999999998</v>
+      </c>
+      <c r="H90" s="5">
+        <v>-74.205699999999993</v>
+      </c>
+      <c r="I90" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J90" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K90" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L90" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A91" s="2">
+        <v>1005823660</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="F91" s="3">
+        <v>26</v>
+      </c>
+      <c r="G91" s="5">
+        <v>4.5871199999999996</v>
+      </c>
+      <c r="H91" s="5">
+        <v>-74.162350000000004</v>
+      </c>
+      <c r="I91" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J91" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K91" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L91" s="3" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A92" s="2">
+        <v>79494633</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D92" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="E92" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="F92" s="3">
+        <v>8</v>
+      </c>
+      <c r="G92" s="5">
+        <v>4.6558000000000002</v>
+      </c>
+      <c r="H92" s="5">
+        <v>-74.074299999999994</v>
+      </c>
+      <c r="I92" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J92" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K92" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L92" s="3" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A93" s="2">
+        <v>1013577097</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="F93" s="3">
+        <v>22</v>
+      </c>
+      <c r="G93" s="5">
+        <v>4.5884600000000004</v>
+      </c>
+      <c r="H93" s="5">
+        <v>-74.195040800000001</v>
+      </c>
+      <c r="I93" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J93" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K93" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L93" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A94" s="2">
+        <v>1010140961</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D94" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="E94" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="F94" s="3">
+        <v>23</v>
+      </c>
+      <c r="G94" s="5">
+        <v>4.6143000000000001</v>
+      </c>
+      <c r="H94" s="5">
+        <v>-74.194500000000005</v>
+      </c>
+      <c r="I94" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J94" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K94" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L94" s="3" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A95" s="2">
+        <v>1030662692</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C95" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="E95" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="F95" s="3">
+        <v>34</v>
+      </c>
+      <c r="G95" s="5">
+        <v>4.6464999999999996</v>
+      </c>
+      <c r="H95" s="5">
+        <v>-74.161199999999994</v>
+      </c>
+      <c r="I95" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J95" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K95" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L95" s="3" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A96" s="2">
+        <v>52505410</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C96" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="F96" s="3">
+        <v>9</v>
+      </c>
+      <c r="G96" s="5">
+        <v>4.5682999999999998</v>
+      </c>
+      <c r="H96" s="5">
+        <v>-74.234300000000005</v>
+      </c>
+      <c r="I96" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J96" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K96" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L96" s="3" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A97" s="2">
+        <v>1033683555</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="F97" s="3">
+        <v>20</v>
+      </c>
+      <c r="G97" s="5">
+        <v>4.5772000000000004</v>
+      </c>
+      <c r="H97" s="5">
+        <v>-74.220100000000002</v>
+      </c>
+      <c r="I97" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J97" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K97" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L97" s="3" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A98" s="2">
+        <v>80722895</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="E98" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="F98" s="3">
+        <v>12</v>
+      </c>
+      <c r="G98" s="5">
+        <v>4.5950452999999998</v>
+      </c>
+      <c r="H98" s="5">
+        <v>-74.194055500000005</v>
+      </c>
+      <c r="I98" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J98" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K98" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L98" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A99" s="2">
+        <v>1031142237</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="E99" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="F99" s="3">
+        <v>25</v>
+      </c>
+      <c r="G99" s="5">
+        <v>4.5512300000000003</v>
+      </c>
+      <c r="H99" s="5">
+        <v>-74.140119999999996</v>
+      </c>
+      <c r="I99" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J99" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K99" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L99" s="3" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A100" s="2">
+        <v>79503448</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="E100" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="F100" s="3">
+        <v>16</v>
+      </c>
+      <c r="G100" s="5">
+        <v>4.6645000000000003</v>
+      </c>
+      <c r="H100" s="5">
+        <v>-74.108199999999997</v>
+      </c>
+      <c r="I100" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J100" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K100" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L100" s="3" t="s">
+        <v>372</v>
       </c>
     </row>
   </sheetData>

</xml_diff>